<commit_message>
older sheets, forgot to commit
</commit_message>
<xml_diff>
--- a/data/VCMRv12.xlsx
+++ b/data/VCMRv12.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\Transcore\New Management\VCMR Repository Documentation\VCMR Spreadsheet for Upload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\data\2023-314-Magnuson_M-VGER-VCMR-website\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28E7643-D49A-4182-8684-44C5FC6330A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93317349-8A98-47A3-AF46-341F9D340FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{DEDBB120-F539-4A49-B84E-9618AC109902}"/>
+    <workbookView xWindow="20760" yWindow="1920" windowWidth="28695" windowHeight="15420" xr2:uid="{DEDBB120-F539-4A49-B84E-9618AC109902}"/>
   </bookViews>
   <sheets>
     <sheet name="VCMRv12" sheetId="1" r:id="rId1"/>
@@ -3639,6 +3639,7 @@
     <col min="1" max="1" width="49.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="255.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>